<commit_message>
Corrige colunas da aba Recusadas do FRADE (categoria/área/alocação)
Planilha fonte corrigida pelo usuário: a aba "Recusadas" do FRADE
tinha as colunas de Categoria/Área Requisitante/Alocação de Custo
desalinhadas, subestimando os valores despriorizados. Total
despriorizado do FRADE passa de US$ 11,2 mi para US$ 22,1 mi,
elevando o total geral despriorizado de US$ 103,3 mi para
US$ 114,2 mi. Recalculado o ranking completo (top 50) e atualizada
a planilha enxuta do FRADE.
</commit_message>
<xml_diff>
--- a/Plano_Integrado_-_FRADE_REV1_enxuta.xlsx
+++ b/Plano_Integrado_-_FRADE_REV1_enxuta.xlsx
@@ -25527,7 +25527,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>70028</v>
+        <v>70000</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -25562,7 +25562,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>70028</v>
+        <v>70000</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -25588,7 +25588,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>70028</v>
+        <v>70000</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -25623,7 +25623,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>70028</v>
+        <v>70000</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -25649,7 +25649,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>255976.36</v>
+        <v>372222</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -25675,19 +25675,19 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>49959.64</v>
+        <v>86295.28</v>
       </c>
       <c r="H4" t="n">
-        <v>52019.36</v>
+        <v>73806.54000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>52018.36</v>
+        <v>73806.54000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>52019.36</v>
+        <v>73806.54000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>49959.64</v>
+        <v>86295.28</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -25710,7 +25710,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3868.72</v>
+        <v>6999.9</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -25760,7 +25760,7 @@
         <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>3868.72</v>
+        <v>6999.9</v>
       </c>
       <c r="P5" t="n">
         <v>0</v>
@@ -25771,7 +25771,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>21.01</v>
+        <v>0.01</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -25797,7 +25797,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -25809,7 +25809,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
@@ -25821,7 +25821,7 @@
         <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>7.01</v>
+        <v>0.01</v>
       </c>
       <c r="P6" t="n">
         <v>0</v>
@@ -25832,7 +25832,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>34739</v>
+        <v>34725</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -25858,7 +25858,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>34739</v>
+        <v>34725</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -25893,7 +25893,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>27013.54</v>
+        <v>26999.54</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -25919,7 +25919,7 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>27013.54</v>
+        <v>26999.54</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -25954,7 +25954,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -25977,7 +25977,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -26015,7 +26015,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -26038,13 +26038,13 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -26076,7 +26076,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -26111,7 +26111,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -26169,7 +26169,7 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>31484.34</v>
+        <v>60430.66</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -26198,7 +26198,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -26251,7 +26251,7 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="Q13" t="n">
         <v>0</v>
@@ -26259,7 +26259,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>25400.62</v>
+        <v>25395.62</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -26291,7 +26291,7 @@
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>12700.31</v>
+        <v>12695.31</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -26309,7 +26309,7 @@
         <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>12700.31</v>
+        <v>12695.31</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
@@ -26352,7 +26352,7 @@
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>30008</v>
+        <v>50000</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -26381,7 +26381,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>71639</v>
+        <v>71619</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -26404,7 +26404,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>71639</v>
+        <v>71619</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -26442,7 +26442,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0</v>
+        <v>880000</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -26465,19 +26465,19 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>220000</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>220000</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>220000</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>220000</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>220000</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -26503,7 +26503,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>26494</v>
+        <v>294981</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -26550,7 +26550,7 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>26494</v>
+        <v>294981</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
@@ -26564,7 +26564,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>448112</v>
+        <v>448028</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -26587,16 +26587,16 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>112028</v>
+        <v>112000</v>
       </c>
       <c r="G19" t="n">
-        <v>112028</v>
+        <v>112000</v>
       </c>
       <c r="H19" t="n">
-        <v>112028</v>
+        <v>112000</v>
       </c>
       <c r="I19" t="n">
-        <v>112028</v>
+        <v>112000</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -26625,7 +26625,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>695220</v>
+        <v>3616292</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -26654,16 +26654,16 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>389476</v>
       </c>
       <c r="I20" t="n">
         <v>307220</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>973691</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>1557905</v>
       </c>
       <c r="L20" t="n">
         <v>0</v>
@@ -26686,7 +26686,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>64575</v>
+        <v>148655</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -26724,10 +26724,10 @@
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>57755</v>
+        <v>57740</v>
       </c>
       <c r="L21" t="n">
-        <v>6820</v>
+        <v>90915</v>
       </c>
       <c r="M21" t="n">
         <v>0</v>
@@ -26747,7 +26747,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>24261.55</v>
+        <v>24254.55</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -26782,7 +26782,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>24261.55</v>
+        <v>24254.55</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -26808,7 +26808,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>9906.379999999999</v>
+        <v>9903.379999999999</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -26831,7 +26831,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>9906.379999999999</v>
+        <v>9903.379999999999</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
@@ -26869,7 +26869,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>483845</v>
+        <v>483510</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -26892,45 +26892,45 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>40321</v>
+        <v>40290</v>
       </c>
       <c r="G24" t="n">
-        <v>40318</v>
+        <v>40290</v>
       </c>
       <c r="H24" t="n">
-        <v>40321</v>
+        <v>40290</v>
       </c>
       <c r="I24" t="n">
-        <v>40320</v>
+        <v>40290</v>
       </c>
       <c r="J24" t="n">
-        <v>40321</v>
+        <v>40290</v>
       </c>
       <c r="K24" t="n">
-        <v>40320</v>
+        <v>40290</v>
       </c>
       <c r="L24" t="n">
-        <v>40321</v>
+        <v>40290</v>
       </c>
       <c r="M24" t="n">
-        <v>40321</v>
+        <v>40290</v>
       </c>
       <c r="N24" t="n">
-        <v>40320</v>
+        <v>40290</v>
       </c>
       <c r="O24" t="n">
-        <v>40321</v>
+        <v>40290</v>
       </c>
       <c r="P24" t="n">
-        <v>40320</v>
+        <v>40290</v>
       </c>
       <c r="Q24" t="n">
-        <v>40321</v>
+        <v>40290</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>271464</v>
+        <v>275433</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -26953,28 +26953,28 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>33933</v>
+        <v>34500</v>
       </c>
       <c r="G25" t="n">
-        <v>33933</v>
+        <v>34500</v>
       </c>
       <c r="H25" t="n">
-        <v>33933</v>
+        <v>34500</v>
       </c>
       <c r="I25" t="n">
-        <v>33933</v>
+        <v>34500</v>
       </c>
       <c r="J25" t="n">
-        <v>33933</v>
+        <v>34500</v>
       </c>
       <c r="K25" t="n">
-        <v>33933</v>
+        <v>34500</v>
       </c>
       <c r="L25" t="n">
-        <v>33933</v>
+        <v>34500</v>
       </c>
       <c r="M25" t="n">
-        <v>33933</v>
+        <v>34500</v>
       </c>
       <c r="N25" t="n">
         <v>0</v>
@@ -26991,7 +26991,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>42014</v>
+        <v>42000</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -27047,12 +27047,12 @@
         <v>0</v>
       </c>
       <c r="Q26" t="n">
-        <v>42014</v>
+        <v>42000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>52514</v>
+        <v>82500</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -27075,7 +27075,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>52514</v>
+        <v>82500</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
@@ -27113,7 +27113,7 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>50028</v>
+        <v>50007</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -27136,7 +27136,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>12507</v>
+        <v>12500</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -27145,7 +27145,7 @@
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>12507</v>
+        <v>12500</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -27154,7 +27154,7 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>12507</v>
+        <v>12500</v>
       </c>
       <c r="M28" t="n">
         <v>0</v>
@@ -27163,7 +27163,7 @@
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>12507</v>
+        <v>12500</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -27174,7 +27174,7 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>250040</v>
+        <v>1020020</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -27200,13 +27200,13 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>645000</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>125020</v>
+        <v>250000</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -27224,7 +27224,7 @@
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>125020</v>
+        <v>250000</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -27235,7 +27235,7 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>250014</v>
+        <v>500000</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -27279,7 +27279,7 @@
         <v>0</v>
       </c>
       <c r="M30" t="n">
-        <v>250014</v>
+        <v>500000</v>
       </c>
       <c r="N30" t="n">
         <v>0</v>
@@ -27296,7 +27296,7 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -27319,7 +27319,7 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="G31" t="n">
         <v>0</v>
@@ -27357,7 +27357,7 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>262027.58</v>
+        <v>321003.4</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -27392,13 +27392,13 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>178664.01</v>
+        <v>178634.01</v>
       </c>
       <c r="K32" t="n">
-        <v>25863.57</v>
+        <v>25858.57</v>
       </c>
       <c r="L32" t="n">
-        <v>33222.22</v>
+        <v>92233.04000000001</v>
       </c>
       <c r="M32" t="n">
         <v>24277.78</v>
@@ -27418,7 +27418,7 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>100014</v>
+        <v>100000</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -27447,7 +27447,7 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>100014</v>
+        <v>100000</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
@@ -27479,7 +27479,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>2400051</v>
+        <v>2700020</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -27508,10 +27508,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>1200031</v>
+        <v>1500000</v>
       </c>
       <c r="I34" t="n">
-        <v>1200020</v>
+        <v>1500000</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -27540,7 +27540,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>126643.22</v>
+        <v>162091.04</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -27587,10 +27587,10 @@
         <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>95279.58</v>
+        <v>95265.58</v>
       </c>
       <c r="O35" t="n">
-        <v>0</v>
+        <v>35461.82</v>
       </c>
       <c r="P35" t="n">
         <v>0</v>
@@ -27601,7 +27601,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>376646.18</v>
+        <v>617060.73</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -27642,13 +27642,13 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>227598.27</v>
+        <v>227568.27</v>
       </c>
       <c r="M36" t="n">
-        <v>75866.08</v>
+        <v>75856.08</v>
       </c>
       <c r="N36" t="n">
-        <v>0</v>
+        <v>240454.55</v>
       </c>
       <c r="O36" t="n">
         <v>0</v>
@@ -27662,7 +27662,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>456692.4000000001</v>
+        <v>456506.4000000001</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -27703,27 +27703,27 @@
         <v>38042.2</v>
       </c>
       <c r="L37" t="n">
-        <v>38073.2</v>
+        <v>38042.2</v>
       </c>
       <c r="M37" t="n">
-        <v>38073.2</v>
+        <v>38042.2</v>
       </c>
       <c r="N37" t="n">
-        <v>38073.2</v>
+        <v>38042.2</v>
       </c>
       <c r="O37" t="n">
-        <v>38073.2</v>
+        <v>38042.2</v>
       </c>
       <c r="P37" t="n">
-        <v>38073.2</v>
+        <v>38042.2</v>
       </c>
       <c r="Q37" t="n">
-        <v>38073.2</v>
+        <v>38042.2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>126042</v>
+        <v>126014</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -27755,7 +27755,7 @@
         <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>42014</v>
+        <v>42000</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -27767,7 +27767,7 @@
         <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>42014</v>
+        <v>42000</v>
       </c>
       <c r="N38" t="n">
         <v>0</v>
@@ -27779,12 +27779,12 @@
         <v>0</v>
       </c>
       <c r="Q38" t="n">
-        <v>42014</v>
+        <v>42000</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>80028</v>
+        <v>80000</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -27813,7 +27813,7 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>40014</v>
+        <v>40000</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
@@ -27834,7 +27834,7 @@
         <v>0</v>
       </c>
       <c r="O39" t="n">
-        <v>40014</v>
+        <v>40000</v>
       </c>
       <c r="P39" t="n">
         <v>0</v>
@@ -27845,7 +27845,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -27868,10 +27868,10 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="G40" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -27906,7 +27906,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>105042</v>
+        <v>105000</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -27947,10 +27947,10 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>70028</v>
+        <v>70000</v>
       </c>
       <c r="M41" t="n">
-        <v>35014</v>
+        <v>35000</v>
       </c>
       <c r="N41" t="n">
         <v>0</v>
@@ -27967,7 +27967,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>105042</v>
+        <v>105000</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -28008,10 +28008,10 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>70028</v>
+        <v>70000</v>
       </c>
       <c r="M42" t="n">
-        <v>35014</v>
+        <v>35000</v>
       </c>
       <c r="N42" t="n">
         <v>0</v>
@@ -28028,7 +28028,7 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>50014</v>
+        <v>350000</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -28057,7 +28057,7 @@
         <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>50014</v>
+        <v>350000</v>
       </c>
       <c r="I43" t="n">
         <v>0</v>
@@ -28089,7 +28089,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>945240</v>
+        <v>1544910</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -28112,45 +28112,45 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>78770</v>
+        <v>138740</v>
       </c>
       <c r="G44" t="n">
-        <v>78770</v>
+        <v>138740</v>
       </c>
       <c r="H44" t="n">
-        <v>78770</v>
+        <v>138740</v>
       </c>
       <c r="I44" t="n">
-        <v>78770</v>
+        <v>138740</v>
       </c>
       <c r="J44" t="n">
-        <v>78770</v>
+        <v>138740</v>
       </c>
       <c r="K44" t="n">
-        <v>78770</v>
+        <v>138740</v>
       </c>
       <c r="L44" t="n">
-        <v>78770</v>
+        <v>138740</v>
       </c>
       <c r="M44" t="n">
-        <v>78770</v>
+        <v>138740</v>
       </c>
       <c r="N44" t="n">
-        <v>78770</v>
+        <v>138740</v>
       </c>
       <c r="O44" t="n">
-        <v>78770</v>
+        <v>138740</v>
       </c>
       <c r="P44" t="n">
-        <v>78770</v>
+        <v>138740</v>
       </c>
       <c r="Q44" t="n">
-        <v>78770</v>
+        <v>78740</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>87556</v>
+        <v>87500</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -28173,10 +28173,10 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>43778</v>
+        <v>43750</v>
       </c>
       <c r="G45" t="n">
-        <v>43778</v>
+        <v>43750</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
@@ -28211,7 +28211,7 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -28258,7 +28258,7 @@
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O46" t="n">
         <v>0</v>
@@ -28272,7 +28272,7 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>309392.47</v>
+        <v>943992.78</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -28295,7 +28295,7 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>309392.47</v>
+        <v>943992.78</v>
       </c>
       <c r="G47" t="n">
         <v>0</v>
@@ -28333,7 +28333,7 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>15013</v>
+        <v>65000</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -28362,7 +28362,7 @@
         <v>0</v>
       </c>
       <c r="H48" t="n">
-        <v>5006</v>
+        <v>5000</v>
       </c>
       <c r="I48" t="n">
         <v>0</v>
@@ -28377,7 +28377,7 @@
         <v>0</v>
       </c>
       <c r="M48" t="n">
-        <v>10007</v>
+        <v>60000</v>
       </c>
       <c r="N48" t="n">
         <v>0</v>
@@ -28394,7 +28394,7 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>54090</v>
+        <v>54030</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -28423,13 +28423,13 @@
         <v>0</v>
       </c>
       <c r="H49" t="n">
-        <v>18030</v>
+        <v>18000</v>
       </c>
       <c r="I49" t="n">
-        <v>18030</v>
+        <v>18000</v>
       </c>
       <c r="J49" t="n">
-        <v>18030</v>
+        <v>18000</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
@@ -28455,7 +28455,7 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>11414</v>
+        <v>11400</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -28493,7 +28493,7 @@
         <v>0</v>
       </c>
       <c r="K50" t="n">
-        <v>11414</v>
+        <v>11400</v>
       </c>
       <c r="L50" t="n">
         <v>0</v>
@@ -28516,7 +28516,7 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>2107</v>
+        <v>2100</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -28539,7 +28539,7 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>2107</v>
+        <v>2100</v>
       </c>
       <c r="G51" t="n">
         <v>0</v>
@@ -28577,7 +28577,7 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>4214</v>
+        <v>4200</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -28615,7 +28615,7 @@
         <v>0</v>
       </c>
       <c r="K52" t="n">
-        <v>4214</v>
+        <v>4200</v>
       </c>
       <c r="L52" t="n">
         <v>0</v>
@@ -28638,7 +28638,7 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>81120</v>
+        <v>81030</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -28661,16 +28661,16 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>18030</v>
+        <v>18000</v>
       </c>
       <c r="G53" t="n">
-        <v>27030</v>
+        <v>27000</v>
       </c>
       <c r="H53" t="n">
-        <v>18030</v>
+        <v>18000</v>
       </c>
       <c r="I53" t="n">
-        <v>18030</v>
+        <v>18000</v>
       </c>
       <c r="J53" t="n">
         <v>0</v>
@@ -28699,7 +28699,7 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>4214</v>
+        <v>4200</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -28734,7 +28734,7 @@
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>4214</v>
+        <v>4200</v>
       </c>
       <c r="K54" t="n">
         <v>0</v>
@@ -28760,7 +28760,7 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>25014</v>
+        <v>50000</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -28810,7 +28810,7 @@
         <v>0</v>
       </c>
       <c r="O55" t="n">
-        <v>25014</v>
+        <v>50000</v>
       </c>
       <c r="P55" t="n">
         <v>0</v>
@@ -28821,7 +28821,7 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>156514</v>
+        <v>156500</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -28871,7 +28871,7 @@
         <v>0</v>
       </c>
       <c r="O56" t="n">
-        <v>26514</v>
+        <v>26500</v>
       </c>
       <c r="P56" t="n">
         <v>0</v>
@@ -28882,7 +28882,7 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>156510</v>
+        <v>156500</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -28926,7 +28926,7 @@
         <v>0</v>
       </c>
       <c r="M57" t="n">
-        <v>26510</v>
+        <v>26500</v>
       </c>
       <c r="N57" t="n">
         <v>0</v>
@@ -28943,7 +28943,7 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>7.01</v>
+        <v>0.01</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -28987,7 +28987,7 @@
         <v>0</v>
       </c>
       <c r="M58" t="n">
-        <v>7.01</v>
+        <v>0.01</v>
       </c>
       <c r="N58" t="n">
         <v>0</v>
@@ -29004,7 +29004,7 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>7.01</v>
+        <v>0.01</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -29042,7 +29042,7 @@
         <v>0</v>
       </c>
       <c r="K59" t="n">
-        <v>7.01</v>
+        <v>0.01</v>
       </c>
       <c r="L59" t="n">
         <v>0</v>
@@ -29065,7 +29065,7 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>14008</v>
+        <v>14000</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -29088,7 +29088,7 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>7004</v>
+        <v>7000</v>
       </c>
       <c r="G60" t="n">
         <v>0</v>
@@ -29109,7 +29109,7 @@
         <v>0</v>
       </c>
       <c r="M60" t="n">
-        <v>7004</v>
+        <v>7000</v>
       </c>
       <c r="N60" t="n">
         <v>0</v>
@@ -29126,7 +29126,7 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>168372</v>
+        <v>168031</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -29149,45 +29149,45 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>14031</v>
+        <v>14000</v>
       </c>
       <c r="G61" t="n">
-        <v>14031</v>
+        <v>14000</v>
       </c>
       <c r="H61" t="n">
-        <v>14031</v>
+        <v>14000</v>
       </c>
       <c r="I61" t="n">
-        <v>14031</v>
+        <v>14000</v>
       </c>
       <c r="J61" t="n">
-        <v>14031</v>
+        <v>14000</v>
       </c>
       <c r="K61" t="n">
-        <v>14031</v>
+        <v>14000</v>
       </c>
       <c r="L61" t="n">
-        <v>14031</v>
+        <v>14000</v>
       </c>
       <c r="M61" t="n">
-        <v>14031</v>
+        <v>14000</v>
       </c>
       <c r="N61" t="n">
-        <v>14031</v>
+        <v>14000</v>
       </c>
       <c r="O61" t="n">
-        <v>14031</v>
+        <v>14000</v>
       </c>
       <c r="P61" t="n">
-        <v>14031</v>
+        <v>14000</v>
       </c>
       <c r="Q61" t="n">
-        <v>14031</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>150042</v>
+        <v>150014</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -29219,7 +29219,7 @@
         <v>0</v>
       </c>
       <c r="I62" t="n">
-        <v>50014</v>
+        <v>50000</v>
       </c>
       <c r="J62" t="n">
         <v>0</v>
@@ -29231,7 +29231,7 @@
         <v>0</v>
       </c>
       <c r="M62" t="n">
-        <v>50014</v>
+        <v>50000</v>
       </c>
       <c r="N62" t="n">
         <v>0</v>
@@ -29243,12 +29243,12 @@
         <v>0</v>
       </c>
       <c r="Q62" t="n">
-        <v>50014</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>40010</v>
+        <v>104000</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -29298,7 +29298,7 @@
         <v>0</v>
       </c>
       <c r="O63" t="n">
-        <v>40010</v>
+        <v>104000</v>
       </c>
       <c r="P63" t="n">
         <v>0</v>
@@ -29309,7 +29309,7 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>177559.78</v>
+        <v>546835.83</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -29353,7 +29353,7 @@
         <v>0</v>
       </c>
       <c r="M64" t="n">
-        <v>177559.78</v>
+        <v>546835.83</v>
       </c>
       <c r="N64" t="n">
         <v>0</v>
@@ -29370,7 +29370,7 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>267028.58</v>
+        <v>876906.9099999999</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -29414,13 +29414,13 @@
         <v>0</v>
       </c>
       <c r="M65" t="n">
-        <v>182371.33</v>
+        <v>182355.33</v>
       </c>
       <c r="N65" t="n">
-        <v>55907.25</v>
+        <v>55901.25</v>
       </c>
       <c r="O65" t="n">
-        <v>0</v>
+        <v>609900.33</v>
       </c>
       <c r="P65" t="n">
         <v>0</v>
@@ -29463,7 +29463,7 @@
         <v>0</v>
       </c>
       <c r="I66" t="n">
-        <v>1.01</v>
+        <v>0.02</v>
       </c>
       <c r="J66" t="n">
         <v>0</v>
@@ -29492,7 +29492,7 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>540014</v>
+        <v>2800721.1</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -29545,7 +29545,7 @@
         <v>0</v>
       </c>
       <c r="P67" t="n">
-        <v>540014</v>
+        <v>2800721.1</v>
       </c>
       <c r="Q67" t="n">
         <v>0</v>
@@ -29553,7 +29553,7 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>150014</v>
+        <v>150000</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -29579,7 +29579,7 @@
         <v>0</v>
       </c>
       <c r="G68" t="n">
-        <v>150014</v>
+        <v>150000</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>
@@ -29614,7 +29614,7 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>103932.17</v>
+        <v>103904.17</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -29667,15 +29667,15 @@
         <v>0</v>
       </c>
       <c r="P69" t="n">
-        <v>3493.22</v>
+        <v>3491.22</v>
       </c>
       <c r="Q69" t="n">
-        <v>88938.95</v>
+        <v>88912.95</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -29713,7 +29713,7 @@
         <v>0</v>
       </c>
       <c r="K70" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L70" t="n">
         <v>0</v>
@@ -29736,7 +29736,7 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>7.01</v>
+        <v>0.01</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -29771,7 +29771,7 @@
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>7.01</v>
+        <v>0.01</v>
       </c>
       <c r="K71" t="n">
         <v>0</v>
@@ -29797,7 +29797,7 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>183804.24</v>
+        <v>191276.94</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -29820,45 +29820,45 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>15317.02</v>
+        <v>16067.29</v>
       </c>
       <c r="G72" t="n">
-        <v>15317.02</v>
+        <v>16067.29</v>
       </c>
       <c r="H72" t="n">
-        <v>15317.02</v>
+        <v>16067.29</v>
       </c>
       <c r="I72" t="n">
-        <v>15317.02</v>
+        <v>16067.29</v>
       </c>
       <c r="J72" t="n">
-        <v>15317.02</v>
+        <v>16067.29</v>
       </c>
       <c r="K72" t="n">
-        <v>15317.02</v>
+        <v>16067.29</v>
       </c>
       <c r="L72" t="n">
-        <v>15317.02</v>
+        <v>16067.29</v>
       </c>
       <c r="M72" t="n">
-        <v>15317.02</v>
+        <v>16067.29</v>
       </c>
       <c r="N72" t="n">
-        <v>15317.02</v>
+        <v>16067.29</v>
       </c>
       <c r="O72" t="n">
-        <v>15317.02</v>
+        <v>16067.29</v>
       </c>
       <c r="P72" t="n">
-        <v>15317.02</v>
+        <v>16067.29</v>
       </c>
       <c r="Q72" t="n">
-        <v>15317.02</v>
+        <v>15287.02</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -29881,10 +29881,10 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G73" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H73" t="n">
         <v>0</v>
@@ -29919,7 +29919,7 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>60022</v>
+        <v>60000</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -29942,7 +29942,7 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>30011</v>
+        <v>30000</v>
       </c>
       <c r="G74" t="n">
         <v>0</v>
@@ -29960,7 +29960,7 @@
         <v>0</v>
       </c>
       <c r="L74" t="n">
-        <v>30011</v>
+        <v>30000</v>
       </c>
       <c r="M74" t="n">
         <v>0</v>
@@ -29980,7 +29980,7 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -30015,10 +30015,10 @@
         <v>0</v>
       </c>
       <c r="J75" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="K75" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="L75" t="n">
         <v>0</v>

</xml_diff>